<commit_message>
Subscription data loader and IPO Listing day cron
</commit_message>
<xml_diff>
--- a/data/Ipo_reports/IPOMatrix_Sample_Reports_2025.xlsx
+++ b/data/Ipo_reports/IPOMatrix_Sample_Reports_2025.xlsx
@@ -5118,13 +5118,13 @@
         <v>37.23</v>
       </c>
       <c r="L56" s="12">
-        <v>54.85</v>
+        <v>53.74</v>
       </c>
       <c r="M56" s="10" t="str">
         <v/>
       </c>
       <c r="N56" s="12">
-        <v>5.48</v>
+        <v>3.35</v>
       </c>
       <c r="O56" s="4" t="str">
         <v/>
@@ -5278,13 +5278,13 @@
         <v>45.44</v>
       </c>
       <c r="L58" s="12">
-        <v>200.9</v>
+        <v>195.1</v>
       </c>
       <c r="M58" s="10" t="str">
         <v/>
       </c>
       <c r="N58" s="12">
-        <v>229.34</v>
+        <v>219.84</v>
       </c>
       <c r="O58" s="4" t="str">
         <v/>
@@ -5358,13 +5358,13 @@
         <v>99.49</v>
       </c>
       <c r="L59" s="12">
-        <v>411.25</v>
+        <v>417.75</v>
       </c>
       <c r="M59" s="10" t="str">
         <v/>
       </c>
       <c r="N59" s="12">
-        <v>383.82</v>
+        <v>391.47</v>
       </c>
       <c r="O59" s="4" t="str">
         <v/>
@@ -5438,13 +5438,13 @@
         <v>16.68</v>
       </c>
       <c r="L60" s="13">
-        <v>186.3</v>
+        <v>202.45</v>
       </c>
       <c r="M60" s="13">
         <v>135.98</v>
       </c>
       <c r="N60" s="13">
-        <v>33.07</v>
+        <v>44.61</v>
       </c>
       <c r="O60" s="4" t="str">
         <v/>
@@ -9669,7 +9669,7 @@
         <v>94.99 (5.54%)</v>
       </c>
       <c r="I113" s="10" t="str">
-        <v>54.00 (-40%)</v>
+        <v>51.36 (-42.93%)</v>
       </c>
       <c r="J113" s="10" t="str">
         <v>100.00 (07-Jan-2026)</v>
@@ -9749,7 +9749,7 @@
         <v>327.80 (88.39%)</v>
       </c>
       <c r="I114" s="10" t="str">
-        <v>280.25 (61.06%)</v>
+        <v>283.00 (62.64%)</v>
       </c>
       <c r="J114" s="10" t="str">
         <v>347.10 (02-Jan-2026)</v>
@@ -9829,7 +9829,7 @@
         <v>151.95 (16.88%)</v>
       </c>
       <c r="I115" s="10" t="str">
-        <v>87.21 (-32.92%)</v>
+        <v>85.23 (-34.44%)</v>
       </c>
       <c r="J115" s="10" t="str">
         <v>156.00 (01-Jan-2026)</v>
@@ -9909,7 +9909,7 @@
         <v>188.20 (1.18%)</v>
       </c>
       <c r="I116" s="10" t="str">
-        <v>208.25 (11.96%)</v>
+        <v>206.20 (10.86%)</v>
       </c>
       <c r="J116" s="10" t="str">
         <v>220.00 (14-Jan-2026)</v>
@@ -9989,7 +9989,7 @@
         <v>200.75 (-16%)</v>
       </c>
       <c r="I117" s="11" t="str">
-        <v>299.90 (25.48%)</v>
+        <v>288.05 (20.52%)</v>
       </c>
       <c r="J117" s="11" t="str">
         <v>315.00 (01-Jun-2026)</v>
@@ -10368,34 +10368,34 @@
         <v>1</v>
       </c>
       <c r="B122" s="10" t="str">
-        <v>Madhusudan Masala Ltd.</v>
+        <v>Sahara Maritime Ltd.</v>
       </c>
       <c r="C122" s="10" t="str">
-        <v>MADHUSUDAN</v>
-      </c>
-      <c r="D122" s="10" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="D122" s="12">
+        <v>544056</v>
       </c>
       <c r="E122" s="10" t="str">
-        <v>NSE</v>
+        <v>BSE</v>
       </c>
       <c r="F122" s="10" t="str">
-        <v>26-Sep-2023</v>
+        <v>26-Dec-2023</v>
       </c>
       <c r="G122" s="12">
-        <v>177.75</v>
+        <v>24.3</v>
       </c>
       <c r="H122" s="12">
-        <v>150</v>
+        <v>20.25</v>
       </c>
       <c r="I122" s="12">
-        <v>27.75</v>
+        <v>4.05</v>
       </c>
       <c r="J122" s="12">
-        <v>18.5</v>
+        <v>20</v>
       </c>
       <c r="K122" s="10" t="str">
-        <v>19 Jun,2026</v>
+        <v>22 Jun,2026</v>
       </c>
       <c r="L122" s="4" t="str">
         <v/>
@@ -10448,34 +10448,34 @@
         <v>2</v>
       </c>
       <c r="B123" s="10" t="str">
-        <v>Repono Ltd.</v>
+        <v>Ashwini Container Movers Ltd.</v>
       </c>
       <c r="C123" s="10" t="str">
-        <v/>
-      </c>
-      <c r="D123" s="12">
-        <v>544463</v>
+        <v>ASHWINI</v>
+      </c>
+      <c r="D123" s="10" t="str">
+        <v/>
       </c>
       <c r="E123" s="10" t="str">
-        <v>BSE</v>
+        <v>NSE</v>
       </c>
       <c r="F123" s="10" t="str">
-        <v>04-Aug-2025</v>
+        <v>19-Dec-2025</v>
       </c>
       <c r="G123" s="12">
-        <v>98.53</v>
+        <v>164.5</v>
       </c>
       <c r="H123" s="12">
-        <v>83.51</v>
+        <v>137.25</v>
       </c>
       <c r="I123" s="12">
-        <v>15.02</v>
+        <v>27.25</v>
       </c>
       <c r="J123" s="12">
-        <v>17.99</v>
+        <v>19.85</v>
       </c>
       <c r="K123" s="10" t="str">
-        <v>19 Jun,2026</v>
+        <v>22 Jun,2026</v>
       </c>
       <c r="L123" s="4" t="str">
         <v/>
@@ -10528,34 +10528,34 @@
         <v>3</v>
       </c>
       <c r="B124" s="10" t="str">
-        <v>Brisk Technovision Ltd.</v>
+        <v>Shri Hare-krishna Sponge Iron Ltd.</v>
       </c>
       <c r="C124" s="10" t="str">
-        <v/>
-      </c>
-      <c r="D124" s="12">
-        <v>544101</v>
+        <v>SHKSIL</v>
+      </c>
+      <c r="D124" s="10" t="str">
+        <v/>
       </c>
       <c r="E124" s="10" t="str">
-        <v>BSE</v>
+        <v>NSE</v>
       </c>
       <c r="F124" s="10" t="str">
-        <v>31-Jan-2024</v>
+        <v>01-Jul-2025</v>
       </c>
       <c r="G124" s="12">
-        <v>93.5</v>
+        <v>41.75</v>
       </c>
       <c r="H124" s="12">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="I124" s="12">
-        <v>11.5</v>
+        <v>6.75</v>
       </c>
       <c r="J124" s="12">
-        <v>14.02</v>
+        <v>19.29</v>
       </c>
       <c r="K124" s="10" t="str">
-        <v>09 Jun,2026</v>
+        <v>22 Jun,2026</v>
       </c>
       <c r="L124" s="4" t="str">
         <v/>
@@ -10608,34 +10608,34 @@
         <v>4</v>
       </c>
       <c r="B125" s="10" t="str">
-        <v>Captain Technocast Ltd.</v>
+        <v>Msafe Equipments Ltd.</v>
       </c>
       <c r="C125" s="10" t="str">
         <v/>
       </c>
       <c r="D125" s="12">
-        <v>540652</v>
+        <v>544695</v>
       </c>
       <c r="E125" s="10" t="str">
         <v>BSE</v>
       </c>
       <c r="F125" s="10" t="str">
-        <v>01-Aug-2017</v>
+        <v>04-Feb-2026</v>
       </c>
       <c r="G125" s="12">
-        <v>238</v>
+        <v>184.75</v>
       </c>
       <c r="H125" s="12">
-        <v>210</v>
+        <v>155.05</v>
       </c>
       <c r="I125" s="12">
-        <v>28</v>
+        <v>29.7</v>
       </c>
       <c r="J125" s="12">
-        <v>13.33</v>
+        <v>19.16</v>
       </c>
       <c r="K125" s="10" t="str">
-        <v>15 Jun,2026</v>
+        <v>22 Jun,2026</v>
       </c>
       <c r="L125" s="4" t="str">
         <v/>
@@ -10688,34 +10688,34 @@
         <v>5</v>
       </c>
       <c r="B126" s="11" t="str">
-        <v>Tgif Agribusiness Ltd.</v>
+        <v>Stanbik Agro Ltd.</v>
       </c>
       <c r="C126" s="11" t="str">
         <v/>
       </c>
       <c r="D126" s="13">
-        <v>544175</v>
+        <v>544659</v>
       </c>
       <c r="E126" s="11" t="str">
         <v>BSE</v>
       </c>
       <c r="F126" s="11" t="str">
-        <v>15-May-2024</v>
+        <v>19-Dec-2025</v>
       </c>
       <c r="G126" s="13">
-        <v>103</v>
+        <v>38.77</v>
       </c>
       <c r="H126" s="13">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="I126" s="13">
-        <v>11</v>
+        <v>5.77</v>
       </c>
       <c r="J126" s="13">
-        <v>11.96</v>
+        <v>17.48</v>
       </c>
       <c r="K126" s="11" t="str">
-        <v>19 Jun,2026</v>
+        <v>22 Jun,2026</v>
       </c>
       <c r="L126" s="4" t="str">
         <v/>
@@ -14226,10 +14226,10 @@
         <v>01-Sep-2025</v>
       </c>
       <c r="H170" s="12">
-        <v>1193</v>
+        <v>1172.25</v>
       </c>
       <c r="I170" s="12">
-        <v>722.76</v>
+        <v>708.45</v>
       </c>
       <c r="J170" s="4" t="str">
         <v/>
@@ -14306,10 +14306,10 @@
         <v>30-Apr-2025</v>
       </c>
       <c r="H171" s="12">
-        <v>1000</v>
+        <v>1019</v>
       </c>
       <c r="I171" s="12">
-        <v>614.29</v>
+        <v>627.86</v>
       </c>
       <c r="J171" s="4" t="str">
         <v/>
@@ -14386,10 +14386,10 @@
         <v>10-Jul-2025</v>
       </c>
       <c r="H172" s="12">
-        <v>274</v>
+        <v>284.85</v>
       </c>
       <c r="I172" s="12">
-        <v>482.98</v>
+        <v>506.06</v>
       </c>
       <c r="J172" s="4" t="str">
         <v/>
@@ -14466,10 +14466,10 @@
         <v>05-Aug-2025</v>
       </c>
       <c r="H173" s="12">
-        <v>3637.8</v>
+        <v>3631.6</v>
       </c>
       <c r="I173" s="12">
-        <v>439.12</v>
+        <v>437.24</v>
       </c>
       <c r="J173" s="4" t="str">
         <v/>
@@ -14546,10 +14546,10 @@
         <v>19-Jun-2025</v>
       </c>
       <c r="H174" s="13">
-        <v>707.65</v>
+        <v>724.9</v>
       </c>
       <c r="I174" s="13">
-        <v>394.86</v>
+        <v>406.92</v>
       </c>
       <c r="J174" s="4" t="str">
         <v/>
@@ -28386,7 +28386,7 @@
         <v>19.41</v>
       </c>
       <c r="H347" s="12">
-        <v>48.63</v>
+        <v>48.85</v>
       </c>
       <c r="I347" s="12">
         <v>27.6</v>
@@ -28466,7 +28466,7 @@
         <v>16.44</v>
       </c>
       <c r="H348" s="12">
-        <v>49.58</v>
+        <v>49.7</v>
       </c>
       <c r="I348" s="12">
         <v>28.06</v>
@@ -28546,7 +28546,7 @@
         <v>13.52</v>
       </c>
       <c r="H349" s="12">
-        <v>32.21</v>
+        <v>33.03</v>
       </c>
       <c r="I349" s="12">
         <v>30.01</v>
@@ -28626,7 +28626,7 @@
         <v>16.55</v>
       </c>
       <c r="H350" s="12">
-        <v>47.89</v>
+        <v>48.04</v>
       </c>
       <c r="I350" s="12">
         <v>34.08</v>
@@ -28706,7 +28706,7 @@
         <v>16.37</v>
       </c>
       <c r="H351" s="13">
-        <v>35.47</v>
+        <v>35.92</v>
       </c>
       <c r="I351" s="13">
         <v>24.68</v>
@@ -29648,22 +29648,22 @@
         <v>2026</v>
       </c>
       <c r="B363" s="12">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C363" s="12">
-        <v>34757.68</v>
+        <v>35691.68</v>
       </c>
       <c r="D363" s="12">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E363" s="12">
-        <v>66</v>
+        <v>66.99</v>
       </c>
       <c r="F363" s="12">
-        <v>10940.4</v>
+        <v>11352.91</v>
       </c>
       <c r="G363" s="12">
-        <v>31.48</v>
+        <v>31.81</v>
       </c>
       <c r="H363" s="4" t="str">
         <v/>
@@ -32558,7 +32558,7 @@
         <v>6.26</v>
       </c>
       <c r="L399" s="12">
-        <v>6.05</v>
+        <v>6.26</v>
       </c>
       <c r="M399" s="4" t="str">
         <v/>
@@ -32605,40 +32605,40 @@
     </row>
     <row r="400" ht="16" customHeight="1">
       <c r="A400" s="10" t="str">
-        <v>Central Mine Planning &amp; Design Institute Ltd.</v>
+        <v>Vegorama Punjabi Angithi Ltd.</v>
       </c>
       <c r="B400" s="10" t="str">
-        <v>Mainboard</v>
+        <v>SME</v>
       </c>
       <c r="C400" s="10" t="str">
-        <v>20-Mar-2026</v>
+        <v>20-May-2026</v>
       </c>
       <c r="D400" s="12">
-        <v>1841.45</v>
+        <v>36.44</v>
       </c>
       <c r="E400" s="12">
-        <v>172</v>
+        <v>77</v>
       </c>
       <c r="F400" s="10" t="str">
-        <v>30-Mar-2026</v>
+        <v>27-May-2026</v>
       </c>
       <c r="G400" s="12">
-        <v>13655250</v>
+        <v>708000</v>
       </c>
       <c r="H400" s="10" t="str">
-        <v>19-Mar-2026</v>
+        <v>19-May-2026</v>
       </c>
       <c r="I400" s="10" t="str">
-        <v>22-Jun-2026</v>
+        <v>23-Jun-2026</v>
       </c>
       <c r="J400" s="12">
-        <v>218.48</v>
+        <v>8.36</v>
       </c>
       <c r="K400" s="12">
-        <v>210.37</v>
+        <v>8.78</v>
       </c>
       <c r="L400" s="12">
-        <v>342.13</v>
+        <v>9.4</v>
       </c>
       <c r="M400" s="4" t="str">
         <v/>
@@ -32685,40 +32685,40 @@
     </row>
     <row r="401" ht="16" customHeight="1">
       <c r="A401" s="10" t="str">
-        <v>Vegorama Punjabi Angithi Ltd.</v>
+        <v>Amir Chand Jagdish Kumar (Exports) Ltd.</v>
       </c>
       <c r="B401" s="10" t="str">
-        <v>SME</v>
+        <v>Mainboard</v>
       </c>
       <c r="C401" s="10" t="str">
-        <v>20-May-2026</v>
+        <v>24-Mar-2026</v>
       </c>
       <c r="D401" s="12">
-        <v>36.44</v>
+        <v>440</v>
       </c>
       <c r="E401" s="12">
-        <v>77</v>
+        <v>212</v>
       </c>
       <c r="F401" s="10" t="str">
-        <v>27-May-2026</v>
+        <v>02-Apr-2026</v>
       </c>
       <c r="G401" s="12">
-        <v>708000</v>
+        <v>1415190</v>
       </c>
       <c r="H401" s="10" t="str">
-        <v>19-May-2026</v>
+        <v>23-Mar-2026</v>
       </c>
       <c r="I401" s="10" t="str">
-        <v>23-Jun-2026</v>
+        <v>27-Jun-2026</v>
       </c>
       <c r="J401" s="12">
-        <v>8.36</v>
+        <v>28.3</v>
       </c>
       <c r="K401" s="12">
-        <v>8.78</v>
+        <v>25.47</v>
       </c>
       <c r="L401" s="12">
-        <v>9.55</v>
+        <v>18.69</v>
       </c>
       <c r="M401" s="4" t="str">
         <v/>
@@ -32765,40 +32765,40 @@
     </row>
     <row r="402" ht="16" customHeight="1">
       <c r="A402" s="10" t="str">
-        <v>Amir Chand Jagdish Kumar (Exports) Ltd.</v>
+        <v>Mehul Telecom Ltd.</v>
       </c>
       <c r="B402" s="10" t="str">
-        <v>Mainboard</v>
+        <v>SME</v>
       </c>
       <c r="C402" s="10" t="str">
-        <v>24-Mar-2026</v>
+        <v>17-Apr-2026</v>
       </c>
       <c r="D402" s="12">
-        <v>440</v>
+        <v>26.32</v>
       </c>
       <c r="E402" s="12">
-        <v>212</v>
+        <v>98</v>
       </c>
       <c r="F402" s="10" t="str">
-        <v>02-Apr-2026</v>
+        <v>24-Apr-2026</v>
       </c>
       <c r="G402" s="12">
-        <v>1415190</v>
+        <v>394800</v>
       </c>
       <c r="H402" s="10" t="str">
-        <v>23-Mar-2026</v>
+        <v>16-Apr-2026</v>
       </c>
       <c r="I402" s="10" t="str">
-        <v>27-Jun-2026</v>
+        <v>21-Jul-2026</v>
       </c>
       <c r="J402" s="12">
-        <v>28.3</v>
+        <v>4.26</v>
       </c>
       <c r="K402" s="12">
-        <v>25.47</v>
+        <v>4.34</v>
       </c>
       <c r="L402" s="12">
-        <v>18.53</v>
+        <v>3.65</v>
       </c>
       <c r="M402" s="4" t="str">
         <v/>
@@ -32878,7 +32878,7 @@
         <v>162.62</v>
       </c>
       <c r="L403" s="13">
-        <v>246.57</v>
+        <v>258.89</v>
       </c>
       <c r="M403" s="4" t="str">
         <v/>
@@ -33488,10 +33488,10 @@
         <v>2026 *</v>
       </c>
       <c r="B411" s="12">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C411" s="12">
-        <v>36960.97</v>
+        <v>37192.94</v>
       </c>
       <c r="D411" s="4" t="str">
         <v/>
@@ -34208,7 +34208,7 @@
         <v>Rs. 0 - 50 cr. - Amount (Rs.cr.)</v>
       </c>
       <c r="B420" s="12">
-        <v>1634</v>
+        <v>1866</v>
       </c>
       <c r="C420" s="12">
         <v>5090</v>
@@ -34288,7 +34288,7 @@
         <v>Rs. 0 - 50 cr. - No. of Issues</v>
       </c>
       <c r="B421" s="12">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C421" s="12">
         <v>183</v>
@@ -34934,22 +34934,22 @@
         <v>3</v>
       </c>
       <c r="D429" s="12">
-        <v>7.63</v>
+        <v>7.58</v>
       </c>
       <c r="E429" s="12">
-        <v>34142.38</v>
+        <v>34374.35</v>
       </c>
       <c r="F429" s="12">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G429" s="12">
-        <v>92.37</v>
+        <v>92.42</v>
       </c>
       <c r="H429" s="12">
-        <v>36960.97</v>
+        <v>37192.94</v>
       </c>
       <c r="I429" s="12">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="J429" s="4" t="str">
         <v/>
@@ -35648,13 +35648,13 @@
         <v>2026</v>
       </c>
       <c r="B438" s="12">
-        <v>36573.95</v>
+        <v>36805.92</v>
       </c>
       <c r="C438" s="12">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D438" s="12">
-        <v>98.95</v>
+        <v>98.96</v>
       </c>
       <c r="E438" s="12">
         <v>387.02</v>
@@ -35663,13 +35663,13 @@
         <v>12</v>
       </c>
       <c r="G438" s="12">
-        <v>1.05</v>
+        <v>1.04</v>
       </c>
       <c r="H438" s="12">
-        <v>36960.97</v>
+        <v>37192.94</v>
       </c>
       <c r="I438" s="12">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="J438" s="4" t="str">
         <v/>
@@ -36368,16 +36368,16 @@
         <v>2026</v>
       </c>
       <c r="B447" s="12">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C447" s="12">
-        <v>23726.78</v>
+        <v>23952.47</v>
       </c>
       <c r="D447" s="12">
-        <v>13234.2</v>
+        <v>13240.48</v>
       </c>
       <c r="E447" s="12">
-        <v>36960.97</v>
+        <v>37192.94</v>
       </c>
       <c r="F447" s="4" t="str">
         <v/>
@@ -37088,10 +37088,10 @@
         <v>2026</v>
       </c>
       <c r="B456" s="12">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C456" s="12">
-        <v>37170.56</v>
+        <v>37414.83</v>
       </c>
       <c r="D456" s="12">
         <v>198.67</v>
@@ -37106,7 +37106,7 @@
         <v/>
       </c>
       <c r="H456" s="12">
-        <v>36960.97</v>
+        <v>37192.94</v>
       </c>
       <c r="I456" s="4" t="str">
         <v/>
@@ -37808,10 +37808,10 @@
         <v>2026</v>
       </c>
       <c r="B465" s="12">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C465" s="12">
-        <v>36960.97</v>
+        <v>37192.94</v>
       </c>
       <c r="D465" s="12">
         <v>193.09</v>
@@ -37823,7 +37823,7 @@
         <v/>
       </c>
       <c r="G465" s="12">
-        <v>36476.56</v>
+        <v>36708.52</v>
       </c>
       <c r="H465" s="4" t="str">
         <v/>
@@ -39485,34 +39485,34 @@
     </row>
     <row r="486" ht="16" customHeight="1">
       <c r="A486" s="10" t="str">
-        <v>Viviana Power Tech Ltd.</v>
+        <v>QMS Medical Allied Services Ltd.</v>
       </c>
       <c r="B486" s="10" t="str">
-        <v>BSE</v>
+        <v>NSE</v>
       </c>
       <c r="C486" s="10" t="str">
         <v/>
       </c>
       <c r="D486" s="10" t="str">
-        <v>VIVIANA</v>
+        <v>QMSMEDI</v>
       </c>
       <c r="E486" s="10" t="str">
-        <v>05-Sep-2022</v>
+        <v>27-Sep-2022</v>
       </c>
       <c r="F486" s="10" t="str">
-        <v>16-Sep-2022</v>
+        <v>11-Oct-2022</v>
       </c>
       <c r="G486" s="10" t="str">
-        <v>01-Jun-2026</v>
+        <v>17-Jun-2026</v>
       </c>
       <c r="H486" s="12">
-        <v>55</v>
+        <v>121</v>
       </c>
       <c r="I486" s="12">
-        <v>94.5</v>
+        <v>134.4</v>
       </c>
       <c r="J486" s="12">
-        <v>813.85</v>
+        <v>107.45</v>
       </c>
       <c r="K486" s="4" t="str">
         <v/>
@@ -39565,34 +39565,34 @@
     </row>
     <row r="487" ht="16" customHeight="1">
       <c r="A487" s="10" t="str">
-        <v>Shanti Educational Initiatives Ltd.</v>
+        <v>Viviana Power Tech Ltd.</v>
       </c>
       <c r="B487" s="10" t="str">
         <v>BSE</v>
       </c>
-      <c r="C487" s="12">
-        <v>539921</v>
+      <c r="C487" s="10" t="str">
+        <v/>
       </c>
       <c r="D487" s="10" t="str">
-        <v>SEIL</v>
+        <v>VIVIANA</v>
       </c>
       <c r="E487" s="10" t="str">
-        <v>01-Jun-2016</v>
+        <v>05-Sep-2022</v>
       </c>
       <c r="F487" s="10" t="str">
-        <v>14-Jun-2016</v>
+        <v>16-Sep-2022</v>
       </c>
       <c r="G487" s="10" t="str">
-        <v>20-Apr-2026</v>
+        <v>01-Jun-2026</v>
       </c>
       <c r="H487" s="12">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="I487" s="12">
-        <v>91</v>
+        <v>94.5</v>
       </c>
       <c r="J487" s="12">
-        <v>203.46</v>
+        <v>851.65</v>
       </c>
       <c r="K487" s="4" t="str">
         <v/>
@@ -39645,34 +39645,34 @@
     </row>
     <row r="488" ht="16" customHeight="1">
       <c r="A488" s="10" t="str">
-        <v>Kwality Pharmaceuticals Ltd.</v>
+        <v>Shanti Educational Initiatives Ltd.</v>
       </c>
       <c r="B488" s="10" t="str">
         <v>BSE</v>
       </c>
       <c r="C488" s="12">
-        <v>539997</v>
+        <v>539921</v>
       </c>
       <c r="D488" s="10" t="str">
-        <v>KPL</v>
+        <v>SEIL</v>
       </c>
       <c r="E488" s="10" t="str">
-        <v>30-Jun-2016</v>
+        <v>01-Jun-2016</v>
       </c>
       <c r="F488" s="10" t="str">
-        <v>18-Jul-2016</v>
+        <v>14-Jun-2016</v>
       </c>
       <c r="G488" s="10" t="str">
         <v>20-Apr-2026</v>
       </c>
       <c r="H488" s="12">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="I488" s="12">
-        <v>44.5</v>
+        <v>91</v>
       </c>
       <c r="J488" s="12">
-        <v>2485.2</v>
+        <v>218.47</v>
       </c>
       <c r="K488" s="4" t="str">
         <v/>
@@ -39725,34 +39725,34 @@
     </row>
     <row r="489" ht="16" customHeight="1">
       <c r="A489" s="10" t="str">
-        <v>RMC Switchgears Ltd.</v>
+        <v>Kwality Pharmaceuticals Ltd.</v>
       </c>
       <c r="B489" s="10" t="str">
         <v>BSE</v>
       </c>
       <c r="C489" s="12">
-        <v>540358</v>
+        <v>539997</v>
       </c>
       <c r="D489" s="10" t="str">
-        <v>RMC</v>
+        <v>KPL</v>
       </c>
       <c r="E489" s="10" t="str">
-        <v>28-Feb-2017</v>
+        <v>30-Jun-2016</v>
       </c>
       <c r="F489" s="10" t="str">
-        <v>14-Mar-2017</v>
+        <v>18-Jul-2016</v>
       </c>
       <c r="G489" s="10" t="str">
-        <v>01-Apr-2026</v>
+        <v>20-Apr-2026</v>
       </c>
       <c r="H489" s="12">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="I489" s="12">
-        <v>32.4</v>
+        <v>44.5</v>
       </c>
       <c r="J489" s="12">
-        <v>312.1</v>
+        <v>2423</v>
       </c>
       <c r="K489" s="4" t="str">
         <v/>
@@ -39805,34 +39805,34 @@
     </row>
     <row r="490" ht="16" customHeight="1">
       <c r="A490" s="11" t="str">
-        <v>BCPL Railway Infrastructure Ltd.</v>
+        <v>RMC Switchgears Ltd.</v>
       </c>
       <c r="B490" s="11" t="str">
         <v>BSE</v>
       </c>
       <c r="C490" s="13">
-        <v>542057</v>
+        <v>540358</v>
       </c>
       <c r="D490" s="11" t="str">
-        <v>BCPL</v>
+        <v>RMC</v>
       </c>
       <c r="E490" s="11" t="str">
-        <v>05-Oct-2018</v>
+        <v>28-Feb-2017</v>
       </c>
       <c r="F490" s="11" t="str">
-        <v>29-Oct-2018</v>
+        <v>14-Mar-2017</v>
       </c>
       <c r="G490" s="11" t="str">
-        <v>27-Mar-2026</v>
+        <v>01-Apr-2026</v>
       </c>
       <c r="H490" s="13">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I490" s="13">
-        <v>36.3</v>
+        <v>32.4</v>
       </c>
       <c r="J490" s="13">
-        <v>75.2</v>
+        <v>359.3</v>
       </c>
       <c r="K490" s="4" t="str">
         <v/>

</xml_diff>